<commit_message>
Rename hardware part numbers: dash to dot separator (152,153,154,155,156,160)
</commit_message>
<xml_diff>
--- a/Screw n thimble.xlsx
+++ b/Screw n thimble.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bc3138b539fcc989/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bc3138b539fcc989/Desktop/SUPERSYSTEMS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="13_ncr:1_{4160BC46-F839-47F7-BCE7-4D63FDD7CF8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF0253DC-14D7-4413-9DC9-335C51707793}"/>
+  <xr:revisionPtr revIDLastSave="51" documentId="13_ncr:1_{4160BC46-F839-47F7-BCE7-4D63FDD7CF8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9293DB8B-B789-407D-9FEF-518F17FDD849}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{10D6525A-E6B5-42F1-9B69-C4143211CA7F}"/>
   </bookViews>
@@ -33,6 +33,28 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -572,7 +594,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94813170-D52D-4C9F-B51B-FAD350529BD0}">
-  <dimension ref="A1:I66"/>
+  <dimension ref="A1:M66"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9.3984375" bestFit="1" customWidth="1"/>
@@ -585,7 +607,7 @@
     <col min="13" max="13" width="13.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -614,7 +636,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -640,7 +662,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -666,7 +688,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -692,7 +714,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -718,7 +740,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -744,7 +766,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -767,7 +789,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -793,7 +815,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -815,8 +837,12 @@
       <c r="I9" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="M9" t="str" cm="1">
+        <f t="array" ref="M9:M17">_xlfn.UNIQUE(A:A)</f>
+        <v>Category</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -838,8 +864,11 @@
       <c r="I10" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="M10" t="str">
+        <v>Screw</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -861,8 +890,11 @@
       <c r="I11" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="M11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -884,8 +916,11 @@
       <c r="I12" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="M12" t="str">
+        <v>Washer</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -910,8 +945,11 @@
       <c r="I13" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="M13" t="str">
+        <v>Grommet</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -936,8 +974,11 @@
       <c r="I14" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="M14" t="str">
+        <v>Spacer</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -959,8 +1000,11 @@
       <c r="I15" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="M15" t="str">
+        <v>Bolt</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -982,8 +1026,11 @@
       <c r="I16" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="M16" t="str">
+        <v>Nut</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -1005,8 +1052,11 @@
       <c r="I17" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="M17" t="str">
+        <v>Thimble</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -1029,7 +1079,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>8</v>
       </c>
@@ -1052,7 +1102,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>8</v>
       </c>
@@ -1078,7 +1128,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>8</v>
       </c>
@@ -1104,7 +1154,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>31</v>
       </c>
@@ -1124,7 +1174,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>31</v>
       </c>
@@ -1144,7 +1194,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>31</v>
       </c>
@@ -1158,7 +1208,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>31</v>
       </c>
@@ -1172,7 +1222,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>31</v>
       </c>
@@ -1186,7 +1236,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>34</v>
       </c>
@@ -1206,7 +1256,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>34</v>
       </c>
@@ -1226,7 +1276,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>38</v>
       </c>

</xml_diff>